<commit_message>
운동DB 작성 1차: EX002~EX006 (확인필요)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135KCav9vVJV3jhFbwUHEXz
</commit_message>
<xml_diff>
--- a/docs/운동DB_설계표.xlsx
+++ b/docs/운동DB_설계표.xlsx
@@ -88,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -110,11 +110,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,6 +189,8 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -549,57 +595,57 @@
           <t>기본정보</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
+      <c r="B1" s="12" t="n"/>
+      <c r="C1" s="12" t="n"/>
+      <c r="D1" s="12" t="n"/>
+      <c r="E1" s="12" t="n"/>
+      <c r="F1" s="13" t="n"/>
       <c r="G1" s="2" t="inlineStr">
         <is>
           <t>해부학</t>
         </is>
       </c>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
+      <c r="H1" s="12" t="n"/>
+      <c r="I1" s="12" t="n"/>
+      <c r="J1" s="13" t="n"/>
       <c r="K1" s="3" t="inlineStr">
         <is>
           <t>역학</t>
         </is>
       </c>
-      <c r="L1" s="3" t="n"/>
-      <c r="M1" s="3" t="n"/>
+      <c r="L1" s="12" t="n"/>
+      <c r="M1" s="13" t="n"/>
       <c r="N1" s="4" t="inlineStr">
         <is>
           <t>설명·처방</t>
         </is>
       </c>
-      <c r="O1" s="4" t="n"/>
-      <c r="P1" s="4" t="n"/>
-      <c r="Q1" s="4" t="n"/>
-      <c r="R1" s="4" t="n"/>
+      <c r="O1" s="12" t="n"/>
+      <c r="P1" s="12" t="n"/>
+      <c r="Q1" s="12" t="n"/>
+      <c r="R1" s="13" t="n"/>
       <c r="S1" s="5" t="inlineStr">
         <is>
           <t>재활·안전</t>
         </is>
       </c>
-      <c r="T1" s="5" t="n"/>
-      <c r="U1" s="5" t="n"/>
+      <c r="T1" s="12" t="n"/>
+      <c r="U1" s="13" t="n"/>
       <c r="V1" s="6" t="inlineStr">
         <is>
           <t>근거</t>
         </is>
       </c>
-      <c r="W1" s="6" t="n"/>
-      <c r="X1" s="6" t="n"/>
-      <c r="Y1" s="6" t="n"/>
-      <c r="Z1" s="6" t="n"/>
+      <c r="W1" s="12" t="n"/>
+      <c r="X1" s="12" t="n"/>
+      <c r="Y1" s="12" t="n"/>
+      <c r="Z1" s="13" t="n"/>
       <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>미디어</t>
         </is>
       </c>
-      <c r="AB1" s="7" t="n"/>
+      <c r="AB1" s="13" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -874,152 +920,635 @@
       <c r="AB3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="n"/>
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>EX002</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>맨몸 스쿼트</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Bodyweight Squat</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>근력, 하체 기능, 체력</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>대퇴사두근, 대둔근 (Escamilla, 2001; Schoenfeld, 2010)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링, 비복근 (Escamilla, 2001)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>고관절·무릎 굴곡/신전, 발목 배측굴곡/저측굴곡, 시상면</t>
+        </is>
+      </c>
       <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
-      <c r="L4" s="9" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>무릎을 굽힐수록 무릎 관절의 압박력·전단력이 커지고, 가장 깊은 지점 근처에서 최대가 된다 (Escamilla, 2001).
+깊이 앉을수록 고관절을 펴는 힘(신전 모멘트)이 커진다 (Schoenfeld, 2010).
+무릎이 발끝보다 크게 앞으로 나가면 무릎 전단력이 커진다. 단, 이를 막으려다 허리·고관절 자세가 무너지면 안 된다 (Schoenfeld, 2010).</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>무릎이 안쪽으로 모임(외반) — 전방십자인대 부담이 커질 수 있음 (Schoenfeld, 2010)
+내려갈 때 발뒤꿈치가 들림 — 발목 유연성을 먼저 기르기 (Schoenfeld, 2010)
+깊이 앉을 때 골반이 뒤로 말림 — 허리 부담 증가 (Schoenfeld, 2010)
+떨어지듯 빠르게 앉음 — 무릎 관절에 걸리는 힘 증가 (Schoenfeld, 2010)</t>
+        </is>
+      </c>
       <c r="M4" s="9" t="n"/>
-      <c r="N4" s="9" t="n"/>
-      <c r="O4" s="9" t="n"/>
-      <c r="P4" s="9" t="n"/>
-      <c r="Q4" s="9" t="n"/>
-      <c r="R4" s="9" t="n"/>
-      <c r="S4" s="9" t="n"/>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>1) 무릎이 발끝과 같은 방향으로 움직이는 편한 너비로 선다
+2) 엉덩이를 뒤로 보내며 앉고, 2~3초에 걸쳐 천천히 내려간다
+3) 허리는 자연스러운 곡선을 유지하고 시선은 정면을 본다
+4) 발뒤꿈치를 바닥에 붙인 채 밀며 일어선다
+(Schoenfeld, 2010)</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>엉덩이·무릎·발목 근육을 한 번에 쓰는 운동으로, 대퇴사두근·햄스트링·비복근이 중간~높은 수준으로 활성화된다 (Escamilla, 2001).
+올바른 자세로 하면 무릎 안정성을 해치지 않고 오히려 높일 수 있다 (Escamilla, 2001).</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>얕게 앉기(무릎 0~50°) — 무릎에 걸리는 힘이 가장 작은 범위 (Escamilla, 2001)</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>고블릿 스쿼트(EX003)</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T4" s="9" t="n"/>
-      <c r="U4" s="9" t="n"/>
-      <c r="V4" s="9" t="n"/>
-      <c r="W4" s="9" t="n"/>
-      <c r="X4" s="9" t="n"/>
+      <c r="U4" s="9" t="inlineStr">
+        <is>
+          <t>무릎뼈(슬개골) 주변 통증이 있으면 깊게 앉지 않는다 (Schoenfeld, 2010).
+지치면 자세가 무너지기 쉬우므로 자세가 흐트러지면 멈춘다 (Schoenfeld, 2010).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V4" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Escamilla, 2001 — Knee biomechanics of the dynamic squat exercise https://doi.org/10.1097/00005768-200101000-00020
+Schoenfeld, 2010 — Squatting kinematics and kinetics and their application to exercise performance https://doi.org/10.1519/JSC.0b013e3181bac2d7</t>
+        </is>
+      </c>
+      <c r="W4" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X4" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y4" s="9" t="n"/>
-      <c r="Z4" s="9" t="n"/>
+      <c r="Z4" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA4" s="9" t="n"/>
       <c r="AB4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>EX003</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>고블릿 스쿼트</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Goblet Squat</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>근력, 근비대, 하체 기능</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>대퇴사두근 (Collins 외, 2021), 대둔근 (Schoenfeld, 2010)</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링 (Collins 외, 2021)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>고관절·무릎 굴곡/신전, 발목 배측굴곡/저측굴곡, 시상면</t>
+        </is>
+      </c>
       <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>랜드마인 스쿼트와 비교하면 수직 방향 부하가 크고 대퇴사두근을 더 집중적으로 쓴다 (Collins 외, 2021).
+스쿼트 공통: 무릎을 굽힐수록 무릎 관절에 걸리는 힘이 커진다 (Escamilla, 2001).</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>무릎이 안쪽으로 모임(외반) — 전방십자인대 부담이 커질 수 있음 (Schoenfeld, 2010)
+내려갈 때 발뒤꿈치가 들림 — 발목 유연성을 먼저 기르기 (Schoenfeld, 2010)
+깊이 앉을 때 골반이 뒤로 말림 — 허리 부담 증가 (Schoenfeld, 2010)
+떨어지듯 빠르게 앉음 — 무릎 관절에 걸리는 힘 증가 (Schoenfeld, 2010)</t>
+        </is>
+      </c>
       <c r="M5" s="9" t="n"/>
-      <c r="N5" s="9" t="n"/>
-      <c r="O5" s="9" t="n"/>
-      <c r="P5" s="9" t="n"/>
-      <c r="Q5" s="9" t="n"/>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>1) 덤벨이나 케틀벨을 두 손으로 잡아 가슴 앞에 붙인다
+2) 이후는 맨몸 스쿼트와 같다
+1) 무릎이 발끝과 같은 방향으로 움직이는 편한 너비로 선다
+2) 엉덩이를 뒤로 보내며 앉고, 2~3초에 걸쳐 천천히 내려간다
+3) 허리는 자연스러운 곡선을 유지하고 시선은 정면을 본다
+4) 발뒤꿈치를 바닥에 붙인 채 밀며 일어선다
+(Schoenfeld, 2010)</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>가슴 앞에 무게를 들어 대퇴사두근에 더 집중하고 수직 부하를 늘릴 수 있다 (Collins 외, 2021).</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>맨몸 스쿼트(EX002)</t>
+        </is>
+      </c>
       <c r="R5" s="9" t="n"/>
-      <c r="S5" s="9" t="n"/>
+      <c r="S5" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T5" s="9" t="n"/>
-      <c r="U5" s="9" t="n"/>
-      <c r="V5" s="9" t="n"/>
-      <c r="W5" s="9" t="n"/>
-      <c r="X5" s="9" t="n"/>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>무릎뼈(슬개골) 주변 통증이 있으면 깊게 앉지 않는다 (Schoenfeld, 2010).
+지치면 자세가 무너지기 쉬우므로 자세가 흐트러지면 멈춘다 (Schoenfeld, 2010).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V5" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Collins 외, 2021 — Differences in Muscle Activity and Kinetics Between the Goblet Squat and Landmine Squat in Men and Women https://doi.org/10.1519/JSC.0000000000004094
+Schoenfeld, 2010 — Squatting kinematics and kinetics and their application to exercise performance https://doi.org/10.1519/JSC.0b013e3181bac2d7
+Escamilla, 2001 — Knee biomechanics of the dynamic squat exercise https://doi.org/10.1097/00005768-200101000-00020</t>
+        </is>
+      </c>
+      <c r="W5" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X5" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y5" s="9" t="n"/>
-      <c r="Z5" s="9" t="n"/>
+      <c r="Z5" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA5" s="9" t="n"/>
       <c r="AB5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>EX004</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>루마니안 데드리프트</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Romanian Deadlift</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>근력, 근비대, 하체 기능</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>중급</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링(반건양근·대퇴이두근) (McAllister 외, 2014), 대둔근 (Dicus 외, 2023)</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>척추기립근, 중둔근, 비복근 (McAllister 외, 2014), 다열근 (Dicus 외, 2023)</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>고관절 굴곡/신전(힙 힌지), 시상면 (Dicus 외, 2023)</t>
+        </is>
+      </c>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>다리를 거의 편 채 고관절을 접었다 펴는 '힌지' 운동이다 (Dicus 외, 2023).
+반건양근이 대퇴이두근보다 더 많이 활성화됐다 (McAllister 외, 2014).</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M6" s="9" t="n"/>
-      <c r="N6" s="9" t="n"/>
-      <c r="O6" s="9" t="n"/>
-      <c r="P6" s="9" t="n"/>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>비교한 햄스트링 운동 중 햄스트링 활동이 가장 높은 축에 속해, 햄스트링을 최대한 쓰고 싶을 때 권장된다 (McAllister 외, 2014).
+허리와 고관절을 펴는 근육(척추기립근·다열근·대둔근·햄스트링)을 함께 쓴다 (Dicus 외, 2023).</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="n"/>
       <c r="R6" s="9" t="n"/>
-      <c r="S6" s="9" t="n"/>
+      <c r="S6" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T6" s="9" t="n"/>
-      <c r="U6" s="9" t="n"/>
-      <c r="V6" s="9" t="n"/>
-      <c r="W6" s="9" t="n"/>
-      <c r="X6" s="9" t="n"/>
+      <c r="U6" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V6" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+McAllister 외, 2014 — Muscle activation during various hamstring exercises https://doi.org/10.1519/JSC.0000000000000302
+Dicus 외, 2023 — A Comparison of Muscle Recruitment Across Three Straight-Legged, Hinge-Pattern Resistance Training Exercises https://doi.org/10.70252/ZAOJ6139</t>
+        </is>
+      </c>
+      <c r="W6" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X6" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y6" s="9" t="n"/>
-      <c r="Z6" s="9" t="n"/>
+      <c r="Z6" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA6" s="9" t="n"/>
       <c r="AB6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>EX005</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>푸시업</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Push-up</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>근력, 상체, 맨몸 운동</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>대흉근, 전삼각근, 상완삼두근 (EMG 측정 근육: Alizadeh 외, 2020) — 주동근 구분 근거 확인필요</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>어깨 수평 굴곡/신전, 팔꿈치 굴곡/신전</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="9" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>손·발 높이에 따라 부하가 달라진다. 발을 상자에 올리면 바닥 반력이 가장 크고, 손을 올리거나 무릎을 대면 가장 작다 (Ebben 외, 2011).</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M7" s="9" t="n"/>
-      <c r="N7" s="9" t="n"/>
-      <c r="O7" s="9" t="n"/>
-      <c r="P7" s="9" t="n"/>
-      <c r="Q7" s="9" t="n"/>
-      <c r="R7" s="9" t="n"/>
-      <c r="S7" s="9" t="n"/>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>근활성도를 벤치프레스와 비슷하게 맞춘 푸시업(밴드로 부하 추가)은 5주 훈련에서 벤치프레스와 비슷한 근력 향상을 보였다 (Calatayud 외, 2015).</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>손을 높은 곳에 짚고 하기, 무릎 대고 하기 (Ebben 외, 2011)</t>
+        </is>
+      </c>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t>발을 높은 곳에 올리고 하기 (Ebben 외, 2011)</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T7" s="9" t="n"/>
-      <c r="U7" s="9" t="n"/>
-      <c r="V7" s="9" t="n"/>
-      <c r="W7" s="9" t="n"/>
-      <c r="X7" s="9" t="n"/>
+      <c r="U7" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V7" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Ebben 외, 2011 — Kinetic analysis of several variations of push-ups https://doi.org/10.1519/JSC.0b013e31820c8587
+Calatayud 외, 2015 — Bench press and push-up at comparable levels of muscle activity results in similar strength gains https://doi.org/10.1519/JSC.0000000000000589
+Alizadeh 외, 2020 — Push-Ups vs. Bench Press Differences in Repetitions and Muscle Activation between Sexes https://pubmed.ncbi.nlm.nih.gov/32390722/</t>
+        </is>
+      </c>
+      <c r="W7" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X7" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y7" s="9" t="n"/>
-      <c r="Z7" s="9" t="n"/>
+      <c r="Z7" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA7" s="9" t="n"/>
       <c r="AB7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>EX006</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>덤벨 벤트오버 로우</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Dumbbell Bent-over Row</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>근력, 근비대, 상체, 자세</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>중급</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>광배근, 등 상부 근육 (Fenwick 외, 2009)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>척추기립근 등 허리 근육 (Fenwick 외, 2009)</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>어깨 신전, 팔꿈치 굴곡 / 고관절 굽힌 자세 유지</t>
+        </is>
+      </c>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>상체를 숙인 자세라 비교한 세 가지 로우 중 허리(요추) 부하가 가장 컸고, 척추 강성도 가장 높았다 (Fenwick 외, 2009).</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M8" s="9" t="n"/>
-      <c r="N8" s="9" t="n"/>
-      <c r="O8" s="9" t="n"/>
-      <c r="P8" s="9" t="n"/>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>등 위쪽부터 아래쪽까지 근육을 좌우 대칭으로 크게 활성화한다 (Fenwick 외, 2009).</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="n"/>
       <c r="R8" s="9" t="n"/>
-      <c r="S8" s="9" t="n"/>
+      <c r="S8" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T8" s="9" t="n"/>
-      <c r="U8" s="9" t="n"/>
-      <c r="V8" s="9" t="n"/>
-      <c r="W8" s="9" t="n"/>
-      <c r="X8" s="9" t="n"/>
+      <c r="U8" s="9" t="inlineStr">
+        <is>
+          <t>허리 부담을 줄이고 싶다면 허리 부하가 가장 낮았던 인버티드 로우를 고려한다 (Fenwick 외, 2009).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V8" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Fenwick 외, 2009 — Comparison of different rowing exercises: trunk muscle activation and lumbar spine motion, load, and stiffness https://doi.org/10.1519/JSC.0b013e3181942019</t>
+        </is>
+      </c>
+      <c r="W8" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X8" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y8" s="9" t="n"/>
-      <c r="Z8" s="9" t="n"/>
+      <c r="Z8" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA8" s="9" t="n"/>
       <c r="AB8" s="9" t="n"/>
     </row>
@@ -4419,7 +4948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4564,6 +5093,303 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1 (지침)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WHO(Bull 외), 2020</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1 (지침)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Escamilla, 2001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Knee biomechanics of the dynamic squat exercise https://doi.org/10.1097/00005768-200101000-00020</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>4 (리뷰)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Schoenfeld, 2010</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Squatting kinematics and kinetics and their application to exercise performance https://doi.org/10.1519/JSC.0b013e3181bac2d7</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4 (리뷰)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Collins 외, 2021</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Differences in Muscle Activity and Kinetics Between the Goblet Squat and Landmine Squat in Men and Women https://doi.org/10.1519/JSC.0000000000004094</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>McAllister 외, 2014</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Muscle activation during various hamstring exercises https://doi.org/10.1519/JSC.0000000000000302</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dicus 외, 2023</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A Comparison of Muscle Recruitment Across Three Straight-Legged, Hinge-Pattern Resistance Training Exercises https://doi.org/10.70252/ZAOJ6139</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ebben 외, 2011</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kinetic analysis of several variations of push-ups https://doi.org/10.1519/JSC.0b013e31820c8587</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Calatayud 외, 2015</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bench press and push-up at comparable levels of muscle activity results in similar strength gains https://doi.org/10.1519/JSC.0000000000000589</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alizadeh 외, 2020</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Push-Ups vs. Bench Press Differences in Repetitions and Muscle Activation between Sexes https://pubmed.ncbi.nlm.nih.gov/32390722/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fenwick 외, 2009</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Comparison of different rowing exercises: trunk muscle activation and lumbar spine motion, load, and stiffness https://doi.org/10.1519/JSC.0b013e3181942019</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
운동DB 작성 2차: EX007~EX011 (확인필요)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135KCav9vVJV3jhFbwUHEXz
</commit_message>
<xml_diff>
--- a/docs/운동DB_설계표.xlsx
+++ b/docs/운동DB_설계표.xlsx
@@ -1553,152 +1553,574 @@
       <c r="AB8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>EX007</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>런지</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Forward Lunge</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>근력, 근비대, 하체 기능</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>대둔근 (Neto 외, 2020), 대퇴사두근(내측광근) (Ekstrom 외, 2007)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링(대퇴이두근) (Farrokhi 외, 2008)</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>앞다리 고관절·무릎 굴곡/신전, 시상면</t>
+        </is>
+      </c>
       <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
-      <c r="L9" s="9" t="n"/>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>상체를 앞으로 숙이고 런지하면 고관절이 더 굽혀지고, 고관절을 펴는 힘(신전 충격량)과 대둔근·대퇴이두근 활성이 커진다 (Farrokhi 외, 2008).
+상체를 뒤로 젖히는 것은 관절 힘이나 근활성을 바꾸지 않았다 (Farrokhi 외, 2008).</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M9" s="9" t="n"/>
-      <c r="N9" s="9" t="n"/>
-      <c r="O9" s="9" t="n"/>
-      <c r="P9" s="9" t="n"/>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>런지는 내측광근을 최대 근수축의 45% 넘게 활성화해 근력 강화에 도움이 될 수 있다 (Ekstrom 외, 2007).
+일반 런지와 인라인 런지 모두 대둔근 활성이 "매우 높음"(최대의 60% 초과)으로 분류됐다 (Neto 외, 2020).</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>주 2회 이상, 주요 근육군을 모두 포함해 높은 노력으로 한다. 높은 노력은 실패 직전 또는 2~3회 여유(RIR)를 남기는 정도이며, 다양한 무게·세트로 달성할 수 있다 (ACSM, 2026).
+운동당 최소 2세트 (ACSM, 2026).
+근력 목적: 세션당 2~3세트, 1RM의 80% 이상에서 효과가 커짐 (ACSM, 2026).
+근비대 목적: 근육군당 주 10세트 이상 (ACSM, 2026).
+성인은 주 2일 이상, 중강도 이상으로 주요 근육군 근력운동 (WHO, 2020).</t>
+        </is>
+      </c>
       <c r="Q9" s="9" t="n"/>
       <c r="R9" s="9" t="n"/>
-      <c r="S9" s="9" t="n"/>
+      <c r="S9" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T9" s="9" t="n"/>
-      <c r="U9" s="9" t="n"/>
-      <c r="V9" s="9" t="n"/>
-      <c r="W9" s="9" t="n"/>
-      <c r="X9" s="9" t="n"/>
+      <c r="U9" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V9" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Currier 외), 2026 — Resistance Training Prescription for Muscle Function, Hypertrophy, and Physical Performance in Healthy Adults https://doi.org/10.1249/MSS.0000000000003897
+WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Ekstrom 외, 2007 — Electromyographic analysis of core trunk, hip, and thigh muscles during 9 rehabilitation exercises https://doi.org/10.2519/jospt.2007.2471
+Neto 외, 2020 — Gluteus Maximus Activation during Common Strength and Hypertrophy Exercises: A Systematic Review https://pubmed.ncbi.nlm.nih.gov/32132843/
+Farrokhi 외, 2008 — Trunk position influences the kinematics, kinetics, and muscle activity of the lead lower extremity during the forward lunge exercise https://doi.org/10.2519/jospt.2008.2634</t>
+        </is>
+      </c>
+      <c r="W9" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X9" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y9" s="9" t="n"/>
-      <c r="Z9" s="9" t="n"/>
+      <c r="Z9" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA9" s="9" t="n"/>
       <c r="AB9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>EX008</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>글루트 브리지</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Glute Bridge</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>엉덩이 근육, 자세, 맨몸 운동</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>대둔근 (Kang 외, 2016)</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>척추기립근 (Kang 외, 2016)</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>고관절 신전, 시상면</t>
+        </is>
+      </c>
       <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>다리를 30° 벌리고(고관절 외전) 브리지를 하면 0°·15°보다 대둔근 활성이 크고, 허리 근육(척추기립근)의 보상 활동과 골반 앞기울기가 줄었다 (Kang 외, 2016).</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>허리 근육으로 들어 올림(척추기립근 보상) — 다리를 30° 벌리면 줄어든다 (Kang 외, 2016)</t>
+        </is>
+      </c>
       <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9" t="n"/>
-      <c r="O10" s="9" t="n"/>
-      <c r="P10" s="9" t="n"/>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>맨몸 브리지는 근활성이 최대의 45% 미만이어서, 근력보다는 지구력·안정화 훈련에 더 적합할 수 있다 (Ekstrom 외, 2007).
+다리 벌림 각도를 바꾸면 허리 근육 대신 대둔근을 골라서 쓰기 쉬워진다 (Kang 외, 2016).</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Q10" s="9" t="n"/>
       <c r="R10" s="9" t="n"/>
-      <c r="S10" s="9" t="n"/>
+      <c r="S10" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T10" s="9" t="n"/>
-      <c r="U10" s="9" t="n"/>
-      <c r="V10" s="9" t="n"/>
-      <c r="W10" s="9" t="n"/>
-      <c r="X10" s="9" t="n"/>
+      <c r="U10" s="9" t="inlineStr">
+        <is>
+          <t>통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V10" s="9" t="inlineStr">
+        <is>
+          <t>Ekstrom 외, 2007 — Electromyographic analysis of core trunk, hip, and thigh muscles during 9 rehabilitation exercises https://doi.org/10.2519/jospt.2007.2471
+Kang 외, 2016 — Modifying the hip abduction angle during bridging exercise can facilitate gluteus maximus activity https://doi.org/10.1016/j.math.2015.12.010</t>
+        </is>
+      </c>
+      <c r="W10" s="9" t="inlineStr">
+        <is>
+          <t>개별논문</t>
+        </is>
+      </c>
+      <c r="X10" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y10" s="9" t="n"/>
-      <c r="Z10" s="9" t="n"/>
+      <c r="Z10" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA10" s="9" t="n"/>
       <c r="AB10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>EX009</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>플랭크</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Plank</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>근력</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>코어, 자세, 맨몸 운동</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>복직근, 외복사근, 하복부 안정근 (Schoenfeld 외, 2014)</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>몸통 중립 유지(등척성)</t>
+        </is>
+      </c>
       <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
-      <c r="L11" s="9" t="n"/>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>지렛대를 길게 한 자세(long lever)와 골반을 뒤로 마는 자세(후방 경사)를 함께 하면 일반 플랭크보다 상복직근·하복부 안정근·외복사근 활성이 커졌다. 두 요소 중 긴 지렛대의 영향이 더 컸다 (Schoenfeld 외, 2014).</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M11" s="9" t="n"/>
-      <c r="N11" s="9" t="n"/>
-      <c r="O11" s="9" t="n"/>
-      <c r="P11" s="9" t="n"/>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>엎드려 팔꿈치와 발끝으로 버티는 자세(prone bridge)는 근활성이 최대의 45% 미만이어서, 근력보다는 지구력·안정화 훈련에 더 적합할 수 있다 (Ekstrom 외, 2007).</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Q11" s="9" t="n"/>
-      <c r="R11" s="9" t="n"/>
-      <c r="S11" s="9" t="n"/>
+      <c r="R11" s="9" t="inlineStr">
+        <is>
+          <t>긴 지렛대 + 골반 후방 경사 플랭크 (Schoenfeld 외, 2014)</t>
+        </is>
+      </c>
+      <c r="S11" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T11" s="9" t="n"/>
-      <c r="U11" s="9" t="n"/>
-      <c r="V11" s="9" t="n"/>
-      <c r="W11" s="9" t="n"/>
-      <c r="X11" s="9" t="n"/>
+      <c r="U11" s="9" t="inlineStr">
+        <is>
+          <t>통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V11" s="9" t="inlineStr">
+        <is>
+          <t>Ekstrom 외, 2007 — Electromyographic analysis of core trunk, hip, and thigh muscles during 9 rehabilitation exercises https://doi.org/10.2519/jospt.2007.2471
+Schoenfeld 외, 2014 — An electromyographic comparison of a modified version of the plank with a long lever and posterior tilt versus the traditional plank exercise https://doi.org/10.1080/14763141.2014.942355</t>
+        </is>
+      </c>
+      <c r="W11" s="9" t="inlineStr">
+        <is>
+          <t>개별논문</t>
+        </is>
+      </c>
+      <c r="X11" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y11" s="9" t="n"/>
-      <c r="Z11" s="9" t="n"/>
+      <c r="Z11" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA11" s="9" t="n"/>
       <c r="AB11" s="9" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>EX010</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>버드독</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Bird Dog</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>균형·기능</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>코어, 허리 안정, 자세</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>대둔근 (Ekstrom 외, 2007), 몸통 신전근 (Callaghan 외, 1998)</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>고관절 신전, 어깨 굴곡 / 척추 중립 유지</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>척추를 고정한 채 다리를 뻗으면 몸통 근육이 좌우 비대칭으로 활동하고, 척추에 걸리는 부하가 줄어든다 (Callaghan 외, 1998).</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M12" s="9" t="n"/>
-      <c r="N12" s="9" t="n"/>
-      <c r="O12" s="9" t="n"/>
-      <c r="P12" s="9" t="n"/>
-      <c r="Q12" s="9" t="n"/>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>다리 뻗기는 척추 부하가 낮고 허리 근육에 주는 자극이 적당해, 허리 펴는 근육을 처음 강화할 때 위험이 낮은 운동이다. 반대쪽 팔을 함께 뻗으면 난이도가 올라간다 (Callaghan 외, 1998).
+엎드려 팔·다리 들기는 대둔근 강화에 도움이 될 수 있다 (Ekstrom 외, 2007).</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>다리만 뻗기 (Callaghan 외, 1998)</t>
+        </is>
+      </c>
       <c r="R12" s="9" t="n"/>
-      <c r="S12" s="9" t="n"/>
+      <c r="S12" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T12" s="9" t="n"/>
-      <c r="U12" s="9" t="n"/>
-      <c r="V12" s="9" t="n"/>
-      <c r="W12" s="9" t="n"/>
-      <c r="X12" s="9" t="n"/>
+      <c r="U12" s="9" t="inlineStr">
+        <is>
+          <t>통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V12" s="9" t="inlineStr">
+        <is>
+          <t>Callaghan 외, 1998 — The relationship between lumbar spine load and muscle activity during extensor exercises https://doi.org/10.1093/ptj/78.1.8
+Ekstrom 외, 2007 — Electromyographic analysis of core trunk, hip, and thigh muscles during 9 rehabilitation exercises https://doi.org/10.2519/jospt.2007.2471</t>
+        </is>
+      </c>
+      <c r="W12" s="9" t="inlineStr">
+        <is>
+          <t>개별논문</t>
+        </is>
+      </c>
+      <c r="X12" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y12" s="9" t="n"/>
-      <c r="Z12" s="9" t="n"/>
+      <c r="Z12" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA12" s="9" t="n"/>
       <c r="AB12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n"/>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>EX011</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>한발 서기</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Single-leg Stance</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>균형·기능</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>균형, 낙상 예방, 노년</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>한 다리 지지, 발목·고관절 자세 조절</t>
+        </is>
+      </c>
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
-      <c r="L13" s="9" t="n"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M13" s="9" t="n"/>
-      <c r="N13" s="9" t="n"/>
-      <c r="O13" s="9" t="n"/>
-      <c r="P13" s="9" t="n"/>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>균형 훈련은 건강한 노인(65세 이상)의 정적·동적 균형과 예상치 못한 흔들림에 대응하는 능력을 높인다 (Lesinski 외, 2015).
+한발 서기 때 몸의 흔들림(압력 중심 이동)은 균형 능력을 재는 지표로 쓰인다 (Lesinski 외, 2015).</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>65세 이상: 기능적 균형·근력 운동을 강조한 복합 신체활동을 주 3일 이상, 중강도 이상으로 한다 (WHO, 2020).
+균형 훈련 전체 기준으로 효과가 가장 컸던 방식: 11~12주, 주 3회, 1회 31~45분, 주당 총 91~120분 (Lesinski 외, 2015).</t>
+        </is>
+      </c>
       <c r="Q13" s="9" t="n"/>
       <c r="R13" s="9" t="n"/>
-      <c r="S13" s="9" t="n"/>
+      <c r="S13" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T13" s="9" t="n"/>
-      <c r="U13" s="9" t="n"/>
-      <c r="V13" s="9" t="n"/>
-      <c r="W13" s="9" t="n"/>
-      <c r="X13" s="9" t="n"/>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V13" s="9" t="inlineStr">
+        <is>
+          <t>WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+Lesinski 외, 2015 — Effects of Balance Training on Balance Performance in Healthy Older Adults: A Systematic Review and Meta-analysis https://doi.org/10.1007/s40279-015-0375-y</t>
+        </is>
+      </c>
+      <c r="W13" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X13" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y13" s="9" t="n"/>
-      <c r="Z13" s="9" t="n"/>
+      <c r="Z13" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA13" s="9" t="n"/>
       <c r="AB13" s="9" t="n"/>
     </row>
@@ -4948,7 +5370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5390,6 +5812,195 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ekstrom 외, 2007</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Electromyographic analysis of core trunk, hip, and thigh muscles during 9 rehabilitation exercises https://doi.org/10.2519/jospt.2007.2471</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Neto 외, 2020</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Gluteus Maximus Activation during Common Strength and Hypertrophy Exercises: A Systematic Review https://pubmed.ncbi.nlm.nih.gov/32132843/</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Farrokhi 외, 2008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Trunk position influences the kinematics, kinetics, and muscle activity of the lead lower extremity during the forward lunge exercise https://doi.org/10.2519/jospt.2008.2634</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kang 외, 2016</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Modifying the hip abduction angle during bridging exercise can facilitate gluteus maximus activity https://doi.org/10.1016/j.math.2015.12.010</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Schoenfeld 외, 2014</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>An electromyographic comparison of a modified version of the plank with a long lever and posterior tilt versus the traditional plank exercise https://doi.org/10.1080/14763141.2014.942355</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Callaghan 외, 1998</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>The relationship between lumbar spine load and muscle activity during extensor exercises https://doi.org/10.1093/ptj/78.1.8</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3 (개별논문)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lesinski 외, 2015</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Effects of Balance Training on Balance Performance in Healthy Older Adults: A Systematic Review and Meta-analysis https://doi.org/10.1007/s40279-015-0375-y</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
운동DB 작성 3차: EX012~EX016 (확인필요)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135KCav9vVJV3jhFbwUHEXz
</commit_message>
<xml_diff>
--- a/docs/운동DB_설계표.xlsx
+++ b/docs/운동DB_설계표.xlsx
@@ -2125,152 +2125,558 @@
       <c r="AB13" s="9" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>EX012</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>빠르게 걷기</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Brisk Walking</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>유산소</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>심폐 체력, 건강 유지</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>보행 (고관절·무릎·발목 굴곡/신전 반복), 시상면</t>
+        </is>
+      </c>
       <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>걷는 속도(분당 걸음 수)와 운동 강도는 밀접하게 관련된다 (Tudor-Locke 외, 2018).</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M14" s="9" t="n"/>
-      <c r="N14" s="9" t="n"/>
-      <c r="O14" s="9" t="n"/>
-      <c r="P14" s="9" t="n"/>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>분당 100걸음 이상으로 걸으면 대체로 중강도(3 METs) 신체활동에 해당한다. 개인차는 있지만 "충분히 빠른 걸음"의 실용적 기준이다 (Tudor-Locke 외, 2018).</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>성인: 중강도 유산소 주 150~300분, 또는 고강도 주 75~150분, 또는 둘을 섞어서 (WHO, 2020).
+중강도는 하루 30분 이상·주 5일 이상(주 150분 이상), 고강도는 하루 20분 이상·주 3일 이상(주 75분 이상) (ACSM, 2011).
+강도 기준: 분당 100걸음 이상 ≈ 중강도 (Tudor-Locke 외, 2018).</t>
+        </is>
+      </c>
       <c r="Q14" s="9" t="n"/>
       <c r="R14" s="9" t="n"/>
-      <c r="S14" s="9" t="n"/>
+      <c r="S14" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T14" s="9" t="n"/>
-      <c r="U14" s="9" t="n"/>
-      <c r="V14" s="9" t="n"/>
-      <c r="W14" s="9" t="n"/>
-      <c r="X14" s="9" t="n"/>
+      <c r="U14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V14" s="9" t="inlineStr">
+        <is>
+          <t>WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Tudor-Locke 외, 2018 — How fast is fast enough? Walking cadence (steps/min) as a practical estimate of intensity in adults https://doi.org/10.1136/bjsports-2017-097628</t>
+        </is>
+      </c>
+      <c r="W14" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X14" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y14" s="9" t="n"/>
-      <c r="Z14" s="9" t="n"/>
+      <c r="Z14" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA14" s="9" t="n"/>
       <c r="AB14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>EX013</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>실내 자전거</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Indoor Cycling</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>유산소</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>심폐 체력, 다이어트, 혈압</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>고관절·무릎 굴곡/신전, 발목 움직임 반복</t>
+        </is>
+      </c>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="n"/>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M15" s="9" t="n"/>
-      <c r="N15" s="9" t="n"/>
-      <c r="O15" s="9" t="n"/>
-      <c r="P15" s="9" t="n"/>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>실내 자전거 운동은 유산소 능력, 혈압, 혈중 지질, 체성분을 개선할 수 있다. 식단 조절과 함께하면 혈중 지질·체중·혈압 개선에 권장된다. 다만 무작위 대조 연구가 적어 신중하게 해석해야 한다 (Chavarrias 외, 2019).</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>성인: 중강도 유산소 주 150~300분, 또는 고강도 주 75~150분, 또는 둘을 섞어서 (WHO, 2020).
+중강도는 하루 30분 이상·주 5일 이상(주 150분 이상), 고강도는 하루 20분 이상·주 3일 이상(주 75분 이상) (ACSM, 2011).</t>
+        </is>
+      </c>
       <c r="Q15" s="9" t="n"/>
       <c r="R15" s="9" t="n"/>
-      <c r="S15" s="9" t="n"/>
+      <c r="S15" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T15" s="9" t="n"/>
-      <c r="U15" s="9" t="n"/>
-      <c r="V15" s="9" t="n"/>
-      <c r="W15" s="9" t="n"/>
-      <c r="X15" s="9" t="n"/>
+      <c r="U15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V15" s="9" t="inlineStr">
+        <is>
+          <t>WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Chavarrias 외, 2019 — Health Benefits of Indoor Cycling: A Systematic Review https://doi.org/10.3390/medicina55080452</t>
+        </is>
+      </c>
+      <c r="W15" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X15" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y15" s="9" t="n"/>
-      <c r="Z15" s="9" t="n"/>
+      <c r="Z15" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA15" s="9" t="n"/>
       <c r="AB15" s="9" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="n"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>EX014</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>줄넘기</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Jump Rope</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>유산소</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>심폐 체력, 순발력, 학교 체육</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>중급</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>발목 저측굴곡 반복 점프</t>
+        </is>
+      </c>
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="9" t="n"/>
-      <c r="L16" s="9" t="n"/>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M16" s="9" t="n"/>
-      <c r="N16" s="9" t="n"/>
-      <c r="O16" s="9" t="n"/>
-      <c r="P16" s="9" t="n"/>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>줄넘기 훈련은 안정시 심박수, 체질량지수, 체지방, 심폐 지구력, 상·하체 최대 근력, 점프, 관절 가동범위, 달리기 속도를 작게~중간 정도 개선했다. 연구 대상은 대부분 18세 미만이다 (Singh 외, 2022).
+10~12세에서는 일반 체육 수업보다 신체 기능·수행 능력 향상 효과가 컸지만, 체형 변화에는 차이가 없었다 (Zhao 외, 2023).</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>어린이·청소년: 하루 평균 60분 이상 중~고강도 신체활동(주로 유산소), 고강도 유산소와 근육·뼈 강화 활동은 주 3일 이상 (WHO, 2020).
+10~12세 줄넘기: 1회 40분 이상, 주 1~2회, 8~12주가 체력 향상에 효과적이었다 (Zhao 외, 2023).
+성인: 성인: 중강도 유산소 주 150~300분, 또는 고강도 주 75~150분, 또는 둘을 섞어서 (WHO, 2020).
+중강도는 하루 30분 이상·주 5일 이상(주 150분 이상), 고강도는 하루 20분 이상·주 3일 이상(주 75분 이상) (ACSM, 2011).</t>
+        </is>
+      </c>
       <c r="Q16" s="9" t="n"/>
       <c r="R16" s="9" t="n"/>
-      <c r="S16" s="9" t="n"/>
+      <c r="S16" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T16" s="9" t="n"/>
-      <c r="U16" s="9" t="n"/>
-      <c r="V16" s="9" t="n"/>
-      <c r="W16" s="9" t="n"/>
-      <c r="X16" s="9" t="n"/>
+      <c r="U16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="V16" s="9" t="inlineStr">
+        <is>
+          <t>WHO(Bull 외), 2020 — WHO 2020 guidelines on physical activity and sedentary behaviour https://doi.org/10.1136/bjsports-2020-102955
+ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Singh 외, 2022 — Jump rope training effects on health- and sport-related physical fitness in young participants: A systematic review with meta-analysis https://doi.org/10.1080/02640414.2022.2099161
+Zhao 외, 2023 — Jumping Rope Improves the Physical Fitness of Preadolescents Aged 10-12 Years: A Meta-Analysis https://doi.org/10.52082/jssm.2023.367</t>
+        </is>
+      </c>
+      <c r="W16" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X16" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y16" s="9" t="n"/>
-      <c r="Z16" s="9" t="n"/>
+      <c r="Z16" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA16" s="9" t="n"/>
       <c r="AB16" s="9" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="9" t="n"/>
-      <c r="I17" s="9" t="n"/>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>EX015</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링 스트레칭</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Hamstring Stretch</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>유연성</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>유연성, 가동범위</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>늘이는 근육: 햄스트링 (Bandy 외, 1997)</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>고관절 굴곡 + 무릎 신전 (햄스트링 신장), 시상면</t>
+        </is>
+      </c>
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="9" t="n"/>
-      <c r="L17" s="9" t="n"/>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M17" s="9" t="n"/>
-      <c r="N17" s="9" t="n"/>
-      <c r="O17" s="9" t="n"/>
-      <c r="P17" s="9" t="n"/>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>햄스트링을 30초 늘려 유지하면 무릎 신전 가동범위가 늘었다. 60초로 늘리거나 하루 3회로 늘려도 효과가 더 커지지 않았다 (Bandy 외, 1997; 21~39세, 주 5일·6주).
+스트레칭 직후 가동범위가 늘어나는 효과는 보통 30분이 안 되게 유지된다 (Behm 외, 2016).</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>주요 근육-힘줄 그룹마다 스트레칭을 합계 60초씩, 주 2일 이상 한다 (ACSM, 2011).
+햄스트링: 한 번에 30초, 하루 1회면 충분했다 (Bandy 외, 1997).</t>
+        </is>
+      </c>
       <c r="Q17" s="9" t="n"/>
       <c r="R17" s="9" t="n"/>
-      <c r="S17" s="9" t="n"/>
+      <c r="S17" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T17" s="9" t="n"/>
-      <c r="U17" s="9" t="n"/>
-      <c r="V17" s="9" t="n"/>
-      <c r="W17" s="9" t="n"/>
-      <c r="X17" s="9" t="n"/>
+      <c r="U17" s="9" t="inlineStr">
+        <is>
+          <t>운동 직전에 한 근육당 60초 이상 정적 스트레칭을 하면 수행력이 조금 떨어질 수 있다(60초 미만은 영향이 더 작음). 스트레칭 뒤 동적 활동을 넣은 준비운동을 권장한다 (Behm 외, 2016).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V17" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Bandy 외, 1997 — The effect of time and frequency of static stretching on flexibility of the hamstring muscles https://doi.org/10.1093/ptj/77.10.1090
+Behm 외, 2016 — Acute effects of muscle stretching on physical performance, range of motion, and injury incidence in healthy active individuals: a systematic review https://doi.org/10.1139/apnm-2015-0235</t>
+        </is>
+      </c>
+      <c r="W17" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X17" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y17" s="9" t="n"/>
-      <c r="Z17" s="9" t="n"/>
+      <c r="Z17" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA17" s="9" t="n"/>
       <c r="AB17" s="9" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="n"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>EX016</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>고관절 굴곡근 스트레칭</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Hip Flexor Stretch</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>유연성</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>유연성, 자세, 가동범위</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>늘이는 근육: 고관절 굴곡근 (Winters 외, 2004)</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>고관절 신전 (고관절 굴곡근 신장), 시상면</t>
+        </is>
+      </c>
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="n"/>
-      <c r="L18" s="9" t="n"/>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M18" s="9" t="n"/>
-      <c r="N18" s="9" t="n"/>
-      <c r="O18" s="9" t="n"/>
-      <c r="P18" s="9" t="n"/>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>고관절 굴곡근이 짧아 고관절 신전이 제한된 사람에게 수동 스트레칭과 능동 스트레칭 모두 6주 동안 가동범위를 비슷하게 늘렸다 (Winters 외, 2004; 허리 통증·하지 손상이 있던 18~25세 대상).</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>주요 근육-힘줄 그룹마다 스트레칭을 합계 60초씩, 주 2일 이상 한다 (ACSM, 2011).</t>
+        </is>
+      </c>
       <c r="Q18" s="9" t="n"/>
       <c r="R18" s="9" t="n"/>
-      <c r="S18" s="9" t="n"/>
+      <c r="S18" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T18" s="9" t="n"/>
-      <c r="U18" s="9" t="n"/>
-      <c r="V18" s="9" t="n"/>
-      <c r="W18" s="9" t="n"/>
-      <c r="X18" s="9" t="n"/>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>운동 직전에 한 근육당 60초 이상 정적 스트레칭을 하면 수행력이 조금 떨어질 수 있다(60초 미만은 영향이 더 작음). 스트레칭 뒤 동적 활동을 넣은 준비운동을 권장한다 (Behm 외, 2016).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V18" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Winters 외, 2004 — Passive versus active stretching of hip flexor muscles in subjects with limited hip extension: a randomized clinical trial https://pubmed.ncbi.nlm.nih.gov/15330693/
+Behm 외, 2016 — Acute effects of muscle stretching on physical performance, range of motion, and injury incidence in healthy active individuals: a systematic review https://doi.org/10.1139/apnm-2015-0235</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X18" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y18" s="9" t="n"/>
-      <c r="Z18" s="9" t="n"/>
+      <c r="Z18" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA18" s="9" t="n"/>
       <c r="AB18" s="9" t="n"/>
     </row>
@@ -5370,7 +5776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6001,6 +6407,222 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ACSM(Garber 외), 2011</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1 (지침)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tudor-Locke 외, 2018</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>How fast is fast enough? Walking cadence (steps/min) as a practical estimate of intensity in adults https://doi.org/10.1136/bjsports-2017-097628</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Chavarrias 외, 2019</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Health Benefits of Indoor Cycling: A Systematic Review https://doi.org/10.3390/medicina55080452</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Singh 외, 2022</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Jump rope training effects on health- and sport-related physical fitness in young participants: A systematic review with meta-analysis https://doi.org/10.1080/02640414.2022.2099161</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Zhao 외, 2023</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Jumping Rope Improves the Physical Fitness of Preadolescents Aged 10-12 Years: A Meta-Analysis https://doi.org/10.52082/jssm.2023.367</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Bandy 외, 1997</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>The effect of time and frequency of static stretching on flexibility of the hamstring muscles https://doi.org/10.1093/ptj/77.10.1090</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Winters 외, 2004</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Passive versus active stretching of hip flexor muscles in subjects with limited hip extension: a randomized clinical trial https://pubmed.ncbi.nlm.nih.gov/15330693/</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Behm 외, 2016</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Acute effects of muscle stretching on physical performance, range of motion, and injury incidence in healthy active individuals: a systematic review https://doi.org/10.1139/apnm-2015-0235</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2 (메타분석·체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>초록 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
운동DB 작성 4차: EX017~EX020 (확인필요)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135KCav9vVJV3jhFbwUHEXz
</commit_message>
<xml_diff>
--- a/docs/운동DB_설계표.xlsx
+++ b/docs/운동DB_설계표.xlsx
@@ -2681,122 +2681,452 @@
       <c r="AB18" s="9" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="9" t="n"/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>EX017</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>흉추 회전 스트레칭</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Thoracic Rotation Stretch</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>유연성</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>유연성, 자세, 거북목</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>흉추 회전, 수평면</t>
+        </is>
+      </c>
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="n"/>
-      <c r="L19" s="9" t="n"/>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M19" s="9" t="n"/>
-      <c r="N19" s="9" t="n"/>
-      <c r="O19" s="9" t="n"/>
-      <c r="P19" s="9" t="n"/>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>거북목 자세와 만성 목 통증이 있는 사람에게 흉추 유연성 운동(주 3일·4주)은 통증, 목·흉추 가동범위, 척추 정렬, 고유감각, 목 장애 지수를 개선했고, 목 안정화 운동보다 효과가 컸다 (Kim &amp; Park, 2026; 24명 대상 소규모 연구).</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>주요 근육-힘줄 그룹마다 스트레칭을 합계 60초씩, 주 2일 이상 한다 (ACSM, 2011).</t>
+        </is>
+      </c>
       <c r="Q19" s="9" t="n"/>
       <c r="R19" s="9" t="n"/>
-      <c r="S19" s="9" t="n"/>
+      <c r="S19" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="T19" s="9" t="n"/>
-      <c r="U19" s="9" t="n"/>
-      <c r="V19" s="9" t="n"/>
-      <c r="W19" s="9" t="n"/>
-      <c r="X19" s="9" t="n"/>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>운동 직전에 한 근육당 60초 이상 정적 스트레칭을 하면 수행력이 조금 떨어질 수 있다. 스트레칭 뒤 동적 활동을 넣은 준비운동을 권장한다 (Behm 외, 2016).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V19" s="9" t="inlineStr">
+        <is>
+          <t>ACSM(Garber 외), 2011 — Quantity and quality of exercise for developing and maintaining cardiorespiratory, musculoskeletal, and neuromotor fitness in apparently healthy adults https://doi.org/10.1249/MSS.0b013e318213fefb
+Kim &amp; Park, 2026 — The Effects of Thoracic Flexibility Exercise on Pain, Range of Motion, Spinal Alignment, Proprioception, and Neck Disability Index in Neck Pain Patients with Forward Head Posture: A Randomized Controlled Trial https://doi.org/10.3390/medicina62091666
+Behm 외, 2016 — Acute effects of muscle stretching on physical performance, range of motion, and injury incidence in healthy active individuals: a systematic review https://doi.org/10.1139/apnm-2015-0235</t>
+        </is>
+      </c>
+      <c r="W19" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X19" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y19" s="9" t="n"/>
-      <c r="Z19" s="9" t="n"/>
+      <c r="Z19" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA19" s="9" t="n"/>
       <c r="AB19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="n"/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>EX018</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>쿼드 세팅</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Quadriceps Setting</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>재활</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>재활, 무릎</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>대퇴사두근 (Alfayyadh, 2026)</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>무릎 신전 방향 등척성 수축</t>
+        </is>
+      </c>
       <c r="J20" s="9" t="n"/>
       <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="n"/>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M20" s="9" t="n"/>
-      <c r="N20" s="9" t="n"/>
-      <c r="O20" s="9" t="n"/>
-      <c r="P20" s="9" t="n"/>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>무릎 수술 후 몇 시간 안에 관절 부기·염증 때문에 대퇴사두근을 마음대로 수축하기 어려워지는 현상(관절성 근억제)이 생긴다. 첫 2주 안에 대응하지 않으면 근력·움직임 결손이 오래 남을 수 있어, 등척성 대퇴사두근 운동 등 초기 활성화 방법이 쓰인다 (Alfayyadh, 2026).
+전방십자인대 재건술 후 첫 2주 동안 대퇴사두근 운동은 안전하게 할 수 있었지만, 가동범위·기능·통증 개선 효과가 임상적으로 크지는 않았다 (Pumell, 2008; 연구 3편).</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Q20" s="9" t="n"/>
       <c r="R20" s="9" t="n"/>
-      <c r="S20" s="9" t="n"/>
-      <c r="T20" s="9" t="n"/>
-      <c r="U20" s="9" t="n"/>
-      <c r="V20" s="9" t="n"/>
-      <c r="W20" s="9" t="n"/>
-      <c r="X20" s="9" t="n"/>
+      <c r="S20" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T20" s="9" t="inlineStr">
+        <is>
+          <t>무릎 수술 후 초기 (근거 연구: 전방십자인대 재건술 후 0~2주)</t>
+        </is>
+      </c>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>수술 후 운동 시작과 진행 일정은 담당 전문가가 정한 일정을 따른다.
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
+          <t>Alfayyadh, 2026 — Early-Phase Quadriceps Activation After Knee Surgery: A Narrative Review https://doi.org/10.3390/jcm15134903
+Pumell, 2008 — Effectiveness of early quadriceps exercises after anterior cruciate ligament reconstruction https://doi.org/10.17159/2078-516X/2008/v20i1a631</t>
+        </is>
+      </c>
+      <c r="W20" s="9" t="inlineStr">
+        <is>
+          <t>개별논문</t>
+        </is>
+      </c>
+      <c r="X20" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y20" s="9" t="n"/>
-      <c r="Z20" s="9" t="n"/>
+      <c r="Z20" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA20" s="9" t="n"/>
       <c r="AB20" s="9" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="9" t="n"/>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>EX019</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>견갑골 후인 운동</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Scapular Retraction Exercise</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>재활</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>재활, 어깨, 자세</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>중부·하부 승모근 (Cools 외, 2007; Cobanoglu 외, 2026)</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>견갑골 후인(모으기)</t>
+        </is>
+      </c>
       <c r="J21" s="9" t="n"/>
-      <c r="K21" s="9" t="n"/>
-      <c r="L21" s="9" t="n"/>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>양쪽 견갑골을 모으며 어깨를 바깥으로 돌리는 운동은 서서 할 때보다 스쿼트 자세로 할 때 중부·하부 승모근 활성이 컸다. 불안정한 바닥에서 스쿼트 자세로 하면 상부 승모근 활성과 비율이 낮아졌다 (Cobanoglu 외, 2026).</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M21" s="9" t="n"/>
-      <c r="N21" s="9" t="n"/>
-      <c r="O21" s="9" t="n"/>
-      <c r="P21" s="9" t="n"/>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>어깨 문제와 관련된 견갑골 근육 불균형 재활에서는 하부·중부 승모근은 많이 쓰고 상부 승모근은 적게 쓰는 운동이 권장된다. 옆으로 누워 바깥돌림, 옆으로 누워 앞으로 들기, 엎드려 수평 벌림+바깥돌림, 엎드려 팔 뒤로 펴기가 이 기준에 가장 적합했다 (Cools 외, 2007).</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Q21" s="9" t="n"/>
       <c r="R21" s="9" t="n"/>
-      <c r="S21" s="9" t="n"/>
-      <c r="T21" s="9" t="n"/>
-      <c r="U21" s="9" t="n"/>
-      <c r="V21" s="9" t="n"/>
-      <c r="W21" s="9" t="n"/>
-      <c r="X21" s="9" t="n"/>
+      <c r="S21" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T21" s="9" t="inlineStr">
+        <is>
+          <t>어깨 (견갑골 주변 근육 불균형)</t>
+        </is>
+      </c>
+      <c r="U21" s="9" t="inlineStr">
+        <is>
+          <t>통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V21" s="9" t="inlineStr">
+        <is>
+          <t>Cools 외, 2007 — Rehabilitation of scapular muscle balance: which exercises to prescribe? https://doi.org/10.1177/0363546507303560
+Cobanoglu 외, 2026 — Trapezius Muscle Activity During Bilateral Scapular Retraction With Shoulder External Rotation https://doi.org/10.1519/JSC.0000000000005631</t>
+        </is>
+      </c>
+      <c r="W21" s="9" t="inlineStr">
+        <is>
+          <t>개별논문</t>
+        </is>
+      </c>
+      <c r="X21" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y21" s="9" t="n"/>
-      <c r="Z21" s="9" t="n"/>
+      <c r="Z21" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA21" s="9" t="n"/>
       <c r="AB21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>EX020</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>종아리 올리기</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Calf Raise (Heel Raise)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>재활</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>재활, 발목, 아킬레스건</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>초급</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>발바닥 굽힘근(종아리 근육) (Chimenti 외, 2024)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>발목 저측굴곡/배측굴곡, 시상면</t>
+        </is>
+      </c>
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="9" t="n"/>
-      <c r="L22" s="9" t="n"/>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="M22" s="9" t="n"/>
-      <c r="N22" s="9" t="n"/>
-      <c r="O22" s="9" t="n"/>
-      <c r="P22" s="9" t="n"/>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>아킬레스건 중간 부위 통증에는 힘줄에 부하를 주는 운동(발바닥 굽힘근의 편심·동심·등척성 수축 등)을 견딜 수 있는 만큼 높은 부하로 하는 것이 1차 방법으로 권고된다. 이런 운동은 기능을 높이고 통증을 줄였다 (Chimenti 외, 2024).
+발뒤꿈치 들기 지구력 검사는 기능 상태를 평가하는 데도 쓰인다 (Chimenti 외, 2024).</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr">
+        <is>
+          <t>주 3회 이상, 견딜 수 있는 만큼 높은 강도로 한다 (Chimenti 외, 2024).</t>
+        </is>
+      </c>
       <c r="Q22" s="9" t="n"/>
       <c r="R22" s="9" t="n"/>
-      <c r="S22" s="9" t="n"/>
-      <c r="T22" s="9" t="n"/>
-      <c r="U22" s="9" t="n"/>
-      <c r="V22" s="9" t="n"/>
-      <c r="W22" s="9" t="n"/>
-      <c r="X22" s="9" t="n"/>
+      <c r="S22" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T22" s="9" t="inlineStr">
+        <is>
+          <t>아킬레스건 중간 부위 통증</t>
+        </is>
+      </c>
+      <c r="U22" s="9" t="inlineStr">
+        <is>
+          <t>증상이 예민한 초기에는 강한 부하를 견디기 어려울 수 있어, 하루 전체 부하를 생각하며 증상 변화에 맞춰 점진적으로 늘린다 (Chimenti 외, 2024).
+힘줄 구조가 약해졌을 가능성이 있는 경우는 위 권고 대상에서 제외된다 (Chimenti 외, 2024).
+통증이 있으면 운동을 멈추고 전문가와 상담하세요.</t>
+        </is>
+      </c>
+      <c r="V22" s="9" t="inlineStr">
+        <is>
+          <t>JOSPT CPG(Chimenti 외), 2024 — Achilles Pain, Stiffness, and Muscle Power Deficits: Midportion Achilles Tendinopathy Revision 2024 https://doi.org/10.2519/jospt.2024.0302</t>
+        </is>
+      </c>
+      <c r="W22" s="9" t="inlineStr">
+        <is>
+          <t>지침</t>
+        </is>
+      </c>
+      <c r="X22" s="9" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
       <c r="Y22" s="9" t="n"/>
-      <c r="Z22" s="9" t="n"/>
+      <c r="Z22" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="AA22" s="9" t="n"/>
       <c r="AB22" s="9" t="n"/>
     </row>
@@ -5776,7 +6106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6623,6 +6953,168 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Kim &amp; Park, 2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>The Effects of Thoracic Flexibility Exercise on Pain, Range of Motion, Spinal Alignment, Proprioception, and Neck Disability Index in Neck Pain Patients with Forward Head Posture: A Randomized Controlled Trial https://doi.org/10.3390/medicina62091666</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Pumell, 2008</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Effectiveness of early quadriceps exercises after anterior cruciate ligament reconstruction https://doi.org/10.17159/2078-516X/2008/v20i1a631</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2 (체계적 고찰)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Alfayyadh, 2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Early-Phase Quadriceps Activation After Knee Surgery: A Narrative Review https://doi.org/10.3390/jcm15134903</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cools 외, 2007</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Rehabilitation of scapular muscle balance: which exercises to prescribe? https://doi.org/10.1177/0363546507303560</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cobanoglu 외, 2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Trapezius Muscle Activity During Bilateral Scapular Retraction With Shoulder External Rotation https://doi.org/10.1519/JSC.0000000000005631</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>3 (개별논문·리뷰)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>JOSPT CPG(Chimenti 외), 2024</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Achilles Pain, Stiffness, and Muscle Power Deficits: Midportion Achilles Tendinopathy Revision 2024 https://doi.org/10.2519/jospt.2024.0302</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1 (지침)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>초록/본문 대조함 (Claude, 2026-10-10). 개발자 검토 필요</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>